<commit_message>
docs(masterplan): correct the Data Out source for A5 and fill the progress grid
</commit_message>
<xml_diff>
--- a/Master Plan API Gateway.xlsx
+++ b/Master Plan API Gateway.xlsx
@@ -76,7 +76,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -129,6 +129,16 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFA0F2D7"/>
         <bgColor rgb="FFA0F2D7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7FEDC8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA0F2D7"/>
       </patternFill>
     </fill>
   </fills>
@@ -349,7 +359,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -471,6 +481,8 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1018,12 +1030,20 @@
         </is>
       </c>
       <c r="H4" s="16" t="n"/>
-      <c r="I4" s="13" t="n"/>
-      <c r="J4" s="16" t="n"/>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="J4" s="16" t="inlineStr">
+        <is>
+          <t>Xong 24/08/2026. Tài liệu triển khai API Gateway + kế hoạch này. 8 agent đã định danh trong dim_agent; ranh giới với dashboard hiện có đã chốt.</t>
+        </is>
+      </c>
       <c r="K4" s="17" t="n"/>
-      <c r="L4" s="17" t="n"/>
-      <c r="M4" s="17" t="n"/>
-      <c r="N4" s="17" t="n"/>
+      <c r="L4" s="53" t="n"/>
+      <c r="M4" s="53" t="n"/>
+      <c r="N4" s="53" t="n"/>
       <c r="O4" s="17" t="n"/>
       <c r="P4" s="17" t="n"/>
       <c r="Q4" s="17" t="n"/>
@@ -1042,9 +1062,9 @@
       <c r="AD4" s="17" t="n"/>
     </row>
     <row r="5" ht="73.5" customHeight="1" s="38">
-      <c r="A5" s="49" t="n"/>
-      <c r="B5" s="49" t="n"/>
-      <c r="C5" s="49" t="n"/>
+      <c r="A5" s="47" t="n"/>
+      <c r="B5" s="47" t="n"/>
+      <c r="C5" s="47" t="n"/>
       <c r="D5" s="14" t="inlineStr">
         <is>
           <t>Đo hiện trạng làm mốc so sánh sau khi có Gateway</t>
@@ -1066,11 +1086,19 @@
         </is>
       </c>
       <c r="H5" s="16" t="n"/>
-      <c r="I5" s="13" t="n"/>
-      <c r="J5" s="16" t="n"/>
+      <c r="I5" s="13" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Xong 21/08/2026. Bộ số nền trước Gateway: 1.189 dòng · 867.657.110 token. Ba nguồn trên fact_usage_daily: billing 708.868.471 · monitoring 450.972.068 · app 110.640.605. Tỷ lệ quy được về người: 12,4%.</t>
+        </is>
+      </c>
       <c r="K5" s="17" t="n"/>
-      <c r="L5" s="17" t="n"/>
-      <c r="M5" s="17" t="n"/>
+      <c r="L5" s="53" t="n"/>
+      <c r="M5" s="53" t="n"/>
       <c r="N5" s="17" t="n"/>
       <c r="O5" s="17" t="n"/>
       <c r="P5" s="17" t="n"/>
@@ -1116,12 +1144,20 @@
       <c r="F6" s="14" t="n"/>
       <c r="G6" s="14" t="n"/>
       <c r="H6" s="16" t="n"/>
-      <c r="I6" s="13" t="n"/>
-      <c r="J6" s="16" t="n"/>
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="J6" s="16" t="inlineStr">
+        <is>
+          <t>Xong 24/08/2026. PostgreSQL 17 (token-ledger-postgres) là engine duy nhất — đường thoát SQLite đã gỡ. Schema do Alembic quản, chỉ tiến không lùi.</t>
+        </is>
+      </c>
       <c r="K6" s="17" t="n"/>
       <c r="L6" s="17" t="n"/>
-      <c r="M6" s="17" t="n"/>
-      <c r="N6" s="17" t="n"/>
+      <c r="M6" s="53" t="n"/>
+      <c r="N6" s="53" t="n"/>
       <c r="O6" s="17" t="n"/>
       <c r="P6" s="17" t="n"/>
       <c r="Q6" s="17" t="n"/>
@@ -1166,14 +1202,23 @@
         </is>
       </c>
       <c r="H7" s="16" t="n"/>
-      <c r="I7" s="13" t="n"/>
-      <c r="J7" s="16" t="n"/>
+      <c r="I7" s="13" t="inlineStr">
+        <is>
+          <t>14/09/2026
+(dự kiến)</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Đang làm. Môi trường ĐO đã dựng được: LiteLLM 1.99.0 (fork litellm_rang_dong, commit f005afa146) trên Docker, 1 tuyến Google AI Studio, trả 200. Còn 7 tuyến còn lại và 3 môi trường.</t>
+        </is>
+      </c>
       <c r="K7" s="17" t="n"/>
       <c r="L7" s="17" t="n"/>
       <c r="M7" s="17" t="n"/>
-      <c r="N7" s="17" t="n"/>
-      <c r="O7" s="17" t="n"/>
-      <c r="P7" s="17" t="n"/>
+      <c r="N7" s="54" t="n"/>
+      <c r="O7" s="54" t="n"/>
+      <c r="P7" s="54" t="n"/>
       <c r="Q7" s="17" t="n"/>
       <c r="R7" s="17" t="n"/>
       <c r="S7" s="17" t="n"/>
@@ -1216,14 +1261,23 @@
         </is>
       </c>
       <c r="H8" s="16" t="n"/>
-      <c r="I8" s="13" t="n"/>
-      <c r="J8" s="16" t="n"/>
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>14/09/2026
+(dự kiến)</t>
+        </is>
+      </c>
+      <c r="J8" s="16" t="inlineStr">
+        <is>
+          <t>Đang làm. 27/08 thêm vào docker-compose.yml (profile gateway): redis 7, 2 instance LiteLLM stateless, nginx làm load balancer, và database litellm riêng trên chính token-ledger-postgres. Chưa nghiệm thu bằng lượt chạy thật.</t>
+        </is>
+      </c>
       <c r="K8" s="17" t="n"/>
       <c r="L8" s="17" t="n"/>
       <c r="M8" s="17" t="n"/>
-      <c r="N8" s="17" t="n"/>
-      <c r="O8" s="17" t="n"/>
-      <c r="P8" s="17" t="n"/>
+      <c r="N8" s="54" t="n"/>
+      <c r="O8" s="54" t="n"/>
+      <c r="P8" s="54" t="n"/>
       <c r="Q8" s="17" t="n"/>
       <c r="R8" s="17" t="n"/>
       <c r="S8" s="17" t="n"/>
@@ -1276,15 +1330,24 @@
         </is>
       </c>
       <c r="H9" s="16" t="n"/>
-      <c r="I9" s="13" t="n"/>
-      <c r="J9" s="16" t="n"/>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>21/09/2026
+(dự kiến)</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>Đang làm. Đã đo được JWT đăng nhập đi qua Gateway nguyên vẹn (260 ký tự, đủ claim). Chưa cấp Virtual Key cho agent nào.</t>
+        </is>
+      </c>
       <c r="K9" s="17" t="n"/>
       <c r="L9" s="17" t="n"/>
       <c r="M9" s="17" t="n"/>
       <c r="N9" s="17" t="n"/>
-      <c r="O9" s="17" t="n"/>
-      <c r="P9" s="17" t="n"/>
-      <c r="Q9" s="17" t="n"/>
+      <c r="O9" s="54" t="n"/>
+      <c r="P9" s="54" t="n"/>
+      <c r="Q9" s="54" t="n"/>
       <c r="R9" s="17" t="n"/>
       <c r="S9" s="17" t="n"/>
       <c r="T9" s="17" t="n"/>
@@ -1324,14 +1387,23 @@
         </is>
       </c>
       <c r="H10" s="16" t="n"/>
-      <c r="I10" s="13" t="n"/>
-      <c r="J10" s="16" t="n"/>
+      <c r="I10" s="13" t="inlineStr">
+        <is>
+          <t>14/09/2026
+(dự kiến)</t>
+        </is>
+      </c>
+      <c r="J10" s="16" t="inlineStr">
+        <is>
+          <t>Đo xong 26/08/2026: header khai ở user_header_name → cột end_user; toàn bộ header → proxy_server_request.metadata.headers (8/8 nguyên văn). Cần chốt: end_user giữ claim sub, không giữ cả chuỗi JWT — vì token đổi mỗi lần đăng nhập thì một người sẽ thành nhiều end_user.</t>
+        </is>
+      </c>
       <c r="K10" s="17" t="n"/>
       <c r="L10" s="17" t="n"/>
       <c r="M10" s="17" t="n"/>
-      <c r="N10" s="17" t="n"/>
-      <c r="O10" s="17" t="n"/>
-      <c r="P10" s="17" t="n"/>
+      <c r="N10" s="54" t="n"/>
+      <c r="O10" s="54" t="n"/>
+      <c r="P10" s="54" t="n"/>
       <c r="Q10" s="17" t="n"/>
       <c r="R10" s="17" t="n"/>
       <c r="S10" s="17" t="n"/>
@@ -1382,15 +1454,24 @@
         </is>
       </c>
       <c r="H11" s="16" t="n"/>
-      <c r="I11" s="13" t="n"/>
-      <c r="J11" s="16" t="n"/>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>21/09/2026
+(dự kiến)</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Đang làm. LiteLLM_SpendLogs có 34 cột, đã chép 4 dòng mẫu ra file. spend dựng lại được đến từng chữ số; Gateway ghi cả request THẤT BẠI nên fact_request bắt buộc có cột status. Còn đối chiếu 26 trường sheet Data Out.</t>
+        </is>
+      </c>
       <c r="K11" s="17" t="n"/>
       <c r="L11" s="17" t="n"/>
       <c r="M11" s="17" t="n"/>
-      <c r="N11" s="17" t="n"/>
-      <c r="O11" s="17" t="n"/>
-      <c r="P11" s="17" t="n"/>
-      <c r="Q11" s="17" t="n"/>
+      <c r="N11" s="54" t="n"/>
+      <c r="O11" s="54" t="n"/>
+      <c r="P11" s="54" t="n"/>
+      <c r="Q11" s="54" t="n"/>
       <c r="R11" s="17" t="n"/>
       <c r="S11" s="17" t="n"/>
       <c r="T11" s="17" t="n"/>
@@ -1431,16 +1512,21 @@
         </is>
       </c>
       <c r="H12" s="16" t="n"/>
-      <c r="I12" s="13" t="n"/>
+      <c r="I12" s="13" t="inlineStr">
+        <is>
+          <t>30/09/2026
+(dự kiến)</t>
+        </is>
+      </c>
       <c r="J12" s="16" t="n"/>
       <c r="K12" s="17" t="n"/>
       <c r="L12" s="17" t="n"/>
       <c r="M12" s="17" t="n"/>
       <c r="N12" s="17" t="n"/>
       <c r="O12" s="17" t="n"/>
-      <c r="P12" s="17" t="n"/>
-      <c r="Q12" s="17" t="n"/>
-      <c r="R12" s="17" t="n"/>
+      <c r="P12" s="54" t="n"/>
+      <c r="Q12" s="54" t="n"/>
+      <c r="R12" s="54" t="n"/>
       <c r="S12" s="17" t="n"/>
       <c r="T12" s="17" t="n"/>
       <c r="U12" s="17" t="n"/>
@@ -1493,16 +1579,25 @@
         </is>
       </c>
       <c r="H13" s="16" t="n"/>
-      <c r="I13" s="13" t="n"/>
-      <c r="J13" s="16" t="n"/>
+      <c r="I13" s="13" t="inlineStr">
+        <is>
+          <t>30/09/2026
+(dự kiến)</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Khung 2 instance LiteLLM + load balancer đã có trong docker-compose.yml từ 27/08. Chưa có máy server thứ hai.</t>
+        </is>
+      </c>
       <c r="K13" s="17" t="n"/>
       <c r="L13" s="17" t="n"/>
       <c r="M13" s="17" t="n"/>
       <c r="N13" s="17" t="n"/>
-      <c r="O13" s="17" t="n"/>
-      <c r="P13" s="17" t="n"/>
-      <c r="Q13" s="17" t="n"/>
-      <c r="R13" s="17" t="n"/>
+      <c r="O13" s="54" t="n"/>
+      <c r="P13" s="54" t="n"/>
+      <c r="Q13" s="54" t="n"/>
+      <c r="R13" s="54" t="n"/>
       <c r="S13" s="17" t="n"/>
       <c r="T13" s="17" t="n"/>
       <c r="U13" s="17" t="n"/>
@@ -1543,7 +1638,12 @@
         </is>
       </c>
       <c r="H14" s="16" t="n"/>
-      <c r="I14" s="13" t="n"/>
+      <c r="I14" s="13" t="inlineStr">
+        <is>
+          <t>07/10/2026
+(dự kiến)</t>
+        </is>
+      </c>
       <c r="J14" s="16" t="n"/>
       <c r="K14" s="17" t="n"/>
       <c r="L14" s="17" t="n"/>
@@ -1551,9 +1651,9 @@
       <c r="N14" s="17" t="n"/>
       <c r="O14" s="17" t="n"/>
       <c r="P14" s="17" t="n"/>
-      <c r="Q14" s="17" t="n"/>
-      <c r="R14" s="17" t="n"/>
-      <c r="S14" s="17" t="n"/>
+      <c r="Q14" s="54" t="n"/>
+      <c r="R14" s="54" t="n"/>
+      <c r="S14" s="54" t="n"/>
       <c r="T14" s="17" t="n"/>
       <c r="U14" s="17" t="n"/>
       <c r="V14" s="17" t="n"/>
@@ -1593,7 +1693,12 @@
         </is>
       </c>
       <c r="H15" s="16" t="n"/>
-      <c r="I15" s="13" t="n"/>
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>14/10/2026
+(dự kiến)</t>
+        </is>
+      </c>
       <c r="J15" s="16" t="n"/>
       <c r="K15" s="17" t="n"/>
       <c r="L15" s="17" t="n"/>
@@ -1602,9 +1707,9 @@
       <c r="O15" s="17" t="n"/>
       <c r="P15" s="17" t="n"/>
       <c r="Q15" s="17" t="n"/>
-      <c r="R15" s="17" t="n"/>
-      <c r="S15" s="17" t="n"/>
-      <c r="T15" s="17" t="n"/>
+      <c r="R15" s="54" t="n"/>
+      <c r="S15" s="54" t="n"/>
+      <c r="T15" s="54" t="n"/>
       <c r="U15" s="17" t="n"/>
       <c r="V15" s="17" t="n"/>
       <c r="W15" s="17" t="n"/>
@@ -1652,16 +1757,25 @@
         </is>
       </c>
       <c r="H16" s="16" t="n"/>
-      <c r="I16" s="13" t="n"/>
-      <c r="J16" s="16" t="n"/>
+      <c r="I16" s="13" t="inlineStr">
+        <is>
+          <t>30/09/2026
+(dự kiến)</t>
+        </is>
+      </c>
+      <c r="J16" s="16" t="inlineStr">
+        <is>
+          <t>Chuẩn bị xong 24/08/2026: 10 chỗ đầu đọc đã hết lọc cứng source='app', hệ thống đón được nguồn thứ tư mà không phải sửa một câu SQL nào. Còn chuyển schema sang v2 (40/45 việc, đang chờ một người khác soát độc lập trước khi chạy).</t>
+        </is>
+      </c>
       <c r="K16" s="17" t="n"/>
       <c r="L16" s="17" t="n"/>
-      <c r="M16" s="17" t="n"/>
-      <c r="N16" s="17" t="n"/>
-      <c r="O16" s="17" t="n"/>
-      <c r="P16" s="17" t="n"/>
-      <c r="Q16" s="17" t="n"/>
-      <c r="R16" s="17" t="n"/>
+      <c r="M16" s="53" t="n"/>
+      <c r="N16" s="53" t="n"/>
+      <c r="O16" s="54" t="n"/>
+      <c r="P16" s="54" t="n"/>
+      <c r="Q16" s="54" t="n"/>
+      <c r="R16" s="54" t="n"/>
       <c r="S16" s="17" t="n"/>
       <c r="T16" s="17" t="n"/>
       <c r="U16" s="17" t="n"/>
@@ -1701,7 +1815,12 @@
         </is>
       </c>
       <c r="H17" s="16" t="n"/>
-      <c r="I17" s="13" t="n"/>
+      <c r="I17" s="13" t="inlineStr">
+        <is>
+          <t>07/10/2026
+(dự kiến)</t>
+        </is>
+      </c>
       <c r="J17" s="16" t="n"/>
       <c r="K17" s="17" t="n"/>
       <c r="L17" s="17" t="n"/>
@@ -1709,9 +1828,9 @@
       <c r="N17" s="17" t="n"/>
       <c r="O17" s="17" t="n"/>
       <c r="P17" s="17" t="n"/>
-      <c r="Q17" s="17" t="n"/>
-      <c r="R17" s="17" t="n"/>
-      <c r="S17" s="17" t="n"/>
+      <c r="Q17" s="54" t="n"/>
+      <c r="R17" s="54" t="n"/>
+      <c r="S17" s="54" t="n"/>
       <c r="T17" s="17" t="n"/>
       <c r="U17" s="17" t="n"/>
       <c r="V17" s="17" t="n"/>
@@ -1749,7 +1868,12 @@
         </is>
       </c>
       <c r="H18" s="16" t="n"/>
-      <c r="I18" s="13" t="n"/>
+      <c r="I18" s="13" t="inlineStr">
+        <is>
+          <t>21/10/2026
+(dự kiến)</t>
+        </is>
+      </c>
       <c r="J18" s="16" t="n"/>
       <c r="K18" s="17" t="n"/>
       <c r="L18" s="17" t="n"/>
@@ -1758,10 +1882,10 @@
       <c r="O18" s="17" t="n"/>
       <c r="P18" s="17" t="n"/>
       <c r="Q18" s="17" t="n"/>
-      <c r="R18" s="17" t="n"/>
-      <c r="S18" s="17" t="n"/>
-      <c r="T18" s="17" t="n"/>
-      <c r="U18" s="17" t="n"/>
+      <c r="R18" s="54" t="n"/>
+      <c r="S18" s="54" t="n"/>
+      <c r="T18" s="54" t="n"/>
+      <c r="U18" s="54" t="n"/>
       <c r="V18" s="17" t="n"/>
       <c r="W18" s="17" t="n"/>
       <c r="X18" s="17" t="n"/>
@@ -1809,7 +1933,12 @@
         </is>
       </c>
       <c r="H19" s="16" t="n"/>
-      <c r="I19" s="13" t="n"/>
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>14/11/2026
+(dự kiến)</t>
+        </is>
+      </c>
       <c r="J19" s="16" t="n"/>
       <c r="K19" s="17" t="n"/>
       <c r="L19" s="17" t="n"/>
@@ -1821,10 +1950,10 @@
       <c r="R19" s="17" t="n"/>
       <c r="S19" s="17" t="n"/>
       <c r="T19" s="17" t="n"/>
-      <c r="U19" s="17" t="n"/>
-      <c r="V19" s="17" t="n"/>
-      <c r="W19" s="17" t="n"/>
-      <c r="X19" s="17" t="n"/>
+      <c r="U19" s="54" t="n"/>
+      <c r="V19" s="54" t="n"/>
+      <c r="W19" s="54" t="n"/>
+      <c r="X19" s="54" t="n"/>
       <c r="Y19" s="17" t="n"/>
       <c r="Z19" s="17" t="n"/>
       <c r="AA19" s="17" t="n"/>
@@ -1858,7 +1987,12 @@
         </is>
       </c>
       <c r="H20" s="16" t="n"/>
-      <c r="I20" s="13" t="n"/>
+      <c r="I20" s="13" t="inlineStr">
+        <is>
+          <t>14/10/2026
+(dự kiến)</t>
+        </is>
+      </c>
       <c r="J20" s="16" t="n"/>
       <c r="K20" s="17" t="n"/>
       <c r="L20" s="17" t="n"/>
@@ -1867,9 +2001,9 @@
       <c r="O20" s="17" t="n"/>
       <c r="P20" s="17" t="n"/>
       <c r="Q20" s="17" t="n"/>
-      <c r="R20" s="17" t="n"/>
-      <c r="S20" s="17" t="n"/>
-      <c r="T20" s="17" t="n"/>
+      <c r="R20" s="54" t="n"/>
+      <c r="S20" s="54" t="n"/>
+      <c r="T20" s="54" t="n"/>
       <c r="U20" s="17" t="n"/>
       <c r="V20" s="17" t="n"/>
       <c r="W20" s="17" t="n"/>
@@ -1907,7 +2041,12 @@
         </is>
       </c>
       <c r="H21" s="16" t="n"/>
-      <c r="I21" s="13" t="n"/>
+      <c r="I21" s="13" t="inlineStr">
+        <is>
+          <t>14/11/2026
+(dự kiến)</t>
+        </is>
+      </c>
       <c r="J21" s="16" t="n"/>
       <c r="K21" s="17" t="n"/>
       <c r="L21" s="17" t="n"/>
@@ -1920,9 +2059,9 @@
       <c r="S21" s="17" t="n"/>
       <c r="T21" s="17" t="n"/>
       <c r="U21" s="17" t="n"/>
-      <c r="V21" s="17" t="n"/>
-      <c r="W21" s="17" t="n"/>
-      <c r="X21" s="17" t="n"/>
+      <c r="V21" s="54" t="n"/>
+      <c r="W21" s="54" t="n"/>
+      <c r="X21" s="54" t="n"/>
       <c r="Y21" s="17" t="n"/>
       <c r="Z21" s="17" t="n"/>
       <c r="AA21" s="17" t="n"/>
@@ -1966,7 +2105,12 @@
         </is>
       </c>
       <c r="H22" s="16" t="n"/>
-      <c r="I22" s="13" t="n"/>
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>21/12/2026
+(dự kiến)</t>
+        </is>
+      </c>
       <c r="J22" s="16" t="n"/>
       <c r="K22" s="17" t="n"/>
       <c r="L22" s="17" t="n"/>
@@ -1982,14 +2126,14 @@
       <c r="V22" s="17" t="n"/>
       <c r="W22" s="17" t="n"/>
       <c r="X22" s="17" t="n"/>
-      <c r="Y22" s="17" t="n"/>
-      <c r="Z22" s="17" t="n"/>
-      <c r="AA22" s="17" t="n"/>
-      <c r="AB22" s="17" t="n"/>
-      <c r="AC22" s="17" t="n"/>
+      <c r="Y22" s="54" t="n"/>
+      <c r="Z22" s="54" t="n"/>
+      <c r="AA22" s="54" t="n"/>
+      <c r="AB22" s="54" t="n"/>
+      <c r="AC22" s="54" t="n"/>
       <c r="AD22" s="17" t="n"/>
     </row>
-    <row r="23" ht="14.25" customHeight="1" s="38">
+    <row r="23" s="38">
       <c r="A23" s="47" t="n"/>
       <c r="B23" s="47" t="n"/>
       <c r="C23" s="47" t="n"/>
@@ -2016,7 +2160,12 @@
         </is>
       </c>
       <c r="H23" s="16" t="n"/>
-      <c r="I23" s="13" t="n"/>
+      <c r="I23" s="13" t="inlineStr">
+        <is>
+          <t>31/12/2026
+(dự kiến)</t>
+        </is>
+      </c>
       <c r="J23" s="16" t="n"/>
       <c r="K23" s="17" t="n"/>
       <c r="L23" s="17" t="n"/>
@@ -2036,8 +2185,8 @@
       <c r="Z23" s="17" t="n"/>
       <c r="AA23" s="17" t="n"/>
       <c r="AB23" s="17" t="n"/>
-      <c r="AC23" s="17" t="n"/>
-      <c r="AD23" s="17" t="n"/>
+      <c r="AC23" s="54" t="n"/>
+      <c r="AD23" s="54" t="n"/>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="38"/>
     <row r="25" ht="15.75" customHeight="1" s="38">
@@ -3038,9 +3187,10 @@
   </sheetData>
   <mergeCells count="39">
     <mergeCell ref="C4:C5"/>
+    <mergeCell ref="W2:Z2"/>
+    <mergeCell ref="B11:B12"/>
     <mergeCell ref="O2:R2"/>
     <mergeCell ref="B2:B3"/>
-    <mergeCell ref="B11:B12"/>
     <mergeCell ref="AA2:AD2"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="F2:F3"/>
@@ -3060,9 +3210,8 @@
     <mergeCell ref="A22:A23"/>
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="B6:B8"/>
-    <mergeCell ref="I2:I3"/>
     <mergeCell ref="S2:V2"/>
-    <mergeCell ref="W2:Z2"/>
+    <mergeCell ref="A11:A12"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="J2:J3"/>
     <mergeCell ref="B4:B5"/>
@@ -3074,7 +3223,7 @@
     <mergeCell ref="K2:N2"/>
     <mergeCell ref="B19:B21"/>
     <mergeCell ref="G2:G3"/>
-    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="I2:I3"/>
     <mergeCell ref="A1:AD1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
@@ -3713,7 +3862,7 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Gateway</t>
+          <t>Dẫn xuất từ Gateway</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
@@ -3721,7 +3870,11 @@
           <t>Cột think trên dashboard</t>
         </is>
       </c>
-      <c r="I16" s="6" t="n"/>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>KHÔNG có cột riêng trong LiteLLM_SpendLogs. Quy tắc dẫn xuất, đo có đối chứng 26/08/2026: metadata.usage_object.completion_tokens_details.reasoning_tokens CÓ khoá ⇒ true; khoá VẮNG MẶT HOÀN TOÀN ⇒ false. Vắng mặt, không phải = 0 — đọc nhầm chỗ này thì mọi request đều thành 'có suy luận'.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="19.5" customHeight="1" s="38">
       <c r="A17" s="3" t="n">
@@ -3750,7 +3903,7 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Gateway</t>
+          <t>Dẫn xuất từ Gateway</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
@@ -3760,7 +3913,7 @@
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>text / image / audio</t>
+          <t>text / image / audio. KHÔNG có cột riêng. Dẫn xuất từ metadata.usage_object.completion_tokens_details.{text,audio,image}_tokens — khoá nào có giá trị thì đó là dạng đầu ra. Đo 26/08/2026: text_tokens = 22.</t>
         </is>
       </c>
     </row>

</xml_diff>